<commit_message>
fixing EW department distinctions
</commit_message>
<xml_diff>
--- a/data/RPRB Rule Set.xlsx
+++ b/data/RPRB Rule Set.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxac\Downloads\AI-Transfer\AI-transfer\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD94CF58-1704-4D1D-901E-72D9EDA78ABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63A31954-D55C-46B0-B8B5-C31AA6A38A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" xr2:uid="{F9C510AA-9C50-4780-99E1-BDBC6FD1F28A}"/>
   </bookViews>
@@ -71,9 +71,6 @@
     <t>4S,5I</t>
   </si>
   <si>
-    <t>6EW</t>
-  </si>
-  <si>
     <t>5E</t>
   </si>
   <si>
@@ -113,12 +110,6 @@
     <t>8W,7E</t>
   </si>
   <si>
-    <t>2EW</t>
-  </si>
-  <si>
-    <t>9EW</t>
-  </si>
-  <si>
     <t>Vascular Surgery</t>
   </si>
   <si>
@@ -132,6 +123,15 @@
   </si>
   <si>
     <t>Norris</t>
+  </si>
+  <si>
+    <t>6E,6W</t>
+  </si>
+  <si>
+    <t>9E,9W</t>
+  </si>
+  <si>
+    <t>2E,2W</t>
   </si>
 </sst>
 </file>
@@ -549,125 +549,125 @@
         <v>9</v>
       </c>
       <c r="D2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>12</v>
-      </c>
-      <c r="G2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>15</v>
       </c>
-      <c r="C3" t="s">
-        <v>16</v>
-      </c>
       <c r="D3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
         <v>10</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>12</v>
-      </c>
-      <c r="F3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" t="s">
         <v>19</v>
       </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
       <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" t="s">
         <v>12</v>
-      </c>
-      <c r="G4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
         <v>21</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>22</v>
       </c>
-      <c r="C5" t="s">
-        <v>23</v>
-      </c>
       <c r="D5" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="G5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
         <v>10</v>
       </c>
-      <c r="E6" t="s">
+      <c r="G6" t="s">
         <v>12</v>
-      </c>
-      <c r="F6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" t="s">
         <v>27</v>
       </c>
-      <c r="B7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" t="s">
-        <v>30</v>
-      </c>
       <c r="G7" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>